<commit_message>
Update firewall request _AZ site.xlsx
add information
</commit_message>
<xml_diff>
--- a/firewall request _AZ site.xlsx
+++ b/firewall request _AZ site.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://scconlineservices-my.sharepoint.com/personal/quyen_nguyenthito_scc_com/Documents/Desktop/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Temp\repository\PJservices_account\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{A5C2462B-0F74-4C2A-97BB-1FD677203607}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B32D98E1-0CB4-470A-B1DA-4BDD295B860C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="FirewallCR" sheetId="1" r:id="rId1"/>
@@ -1795,8 +1795,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="Table1" displayName="Table1" ref="A7:M29" totalsRowShown="0">
-  <autoFilter ref="A7:M29" xr:uid="{00000000-0009-0000-0100-000001000000}">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="Table1" displayName="Table1" ref="A7:M30" totalsRowShown="0">
+  <autoFilter ref="A7:M30" xr:uid="{00000000-0009-0000-0100-000001000000}">
     <filterColumn colId="0" hiddenButton="1"/>
     <filterColumn colId="1" hiddenButton="1"/>
     <filterColumn colId="2" hiddenButton="1"/>
@@ -2707,12 +2707,16 @@
       </c>
     </row>
     <row r="30" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="B30" s="15"/>
-      <c r="C30" s="15"/>
-      <c r="D30" s="15"/>
+      <c r="A30" s="1"/>
+      <c r="B30" s="14">
+        <v>124423</v>
+      </c>
+      <c r="C30" s="14"/>
+      <c r="D30" s="14"/>
       <c r="E30" s="14"/>
-      <c r="F30" s="15"/>
+      <c r="F30" s="14"/>
       <c r="G30" s="15"/>
+      <c r="I30" s="1"/>
       <c r="K30" s="15"/>
     </row>
     <row r="31" spans="1:11" x14ac:dyDescent="0.25">
@@ -4033,7 +4037,7 @@
           <x14:formula1>
             <xm:f>Lookup!$A:$A</xm:f>
           </x14:formula1>
-          <xm:sqref>L8:L29</xm:sqref>
+          <xm:sqref>L8:L30</xm:sqref>
         </x14:dataValidation>
       </x14:dataValidations>
     </ext>

</xml_diff>

<commit_message>
Revert "Update firewall request _AZ site.xlsx"
This reverts commit a77d151bc993ffaefeab83769f3c2272a2ad51c6.
</commit_message>
<xml_diff>
--- a/firewall request _AZ site.xlsx
+++ b/firewall request _AZ site.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Temp\repository\PJservices_account\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://scconlineservices-my.sharepoint.com/personal/quyen_nguyenthito_scc_com/Documents/Desktop/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B32D98E1-0CB4-470A-B1DA-4BDD295B860C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{A5C2462B-0F74-4C2A-97BB-1FD677203607}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="FirewallCR" sheetId="1" r:id="rId1"/>
@@ -1795,8 +1795,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="Table1" displayName="Table1" ref="A7:M30" totalsRowShown="0">
-  <autoFilter ref="A7:M30" xr:uid="{00000000-0009-0000-0100-000001000000}">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="Table1" displayName="Table1" ref="A7:M29" totalsRowShown="0">
+  <autoFilter ref="A7:M29" xr:uid="{00000000-0009-0000-0100-000001000000}">
     <filterColumn colId="0" hiddenButton="1"/>
     <filterColumn colId="1" hiddenButton="1"/>
     <filterColumn colId="2" hiddenButton="1"/>
@@ -2707,16 +2707,12 @@
       </c>
     </row>
     <row r="30" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A30" s="1"/>
-      <c r="B30" s="14">
-        <v>124423</v>
-      </c>
-      <c r="C30" s="14"/>
-      <c r="D30" s="14"/>
+      <c r="B30" s="15"/>
+      <c r="C30" s="15"/>
+      <c r="D30" s="15"/>
       <c r="E30" s="14"/>
-      <c r="F30" s="14"/>
+      <c r="F30" s="15"/>
       <c r="G30" s="15"/>
-      <c r="I30" s="1"/>
       <c r="K30" s="15"/>
     </row>
     <row r="31" spans="1:11" x14ac:dyDescent="0.25">
@@ -4037,7 +4033,7 @@
           <x14:formula1>
             <xm:f>Lookup!$A:$A</xm:f>
           </x14:formula1>
-          <xm:sqref>L8:L30</xm:sqref>
+          <xm:sqref>L8:L29</xm:sqref>
         </x14:dataValidation>
       </x14:dataValidations>
     </ext>

</xml_diff>